<commit_message>
Refactor ability score generation and improve character display
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rabbi\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rabbi\Documents\oop-lab\DND_Character_Creator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6B38DB-8F13-4402-86BA-65FC6B9B8E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5CAA011-3134-4501-B715-495026E6A37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RACE" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="102">
   <si>
     <t>key</t>
   </si>
@@ -329,6 +329,9 @@
   </si>
   <si>
     <t>CHA:2</t>
+  </si>
+  <si>
+    <t>hit_die</t>
   </si>
 </sst>
 </file>
@@ -799,13 +802,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DDDB473-1AF9-4E54-9065-790503642D74}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="6" width="13" customWidth="1"/>
+    <col min="1" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="23.06640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -824,8 +828,11 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -844,8 +851,11 @@
       <c r="F2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -864,8 +874,11 @@
       <c r="F3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -884,8 +897,11 @@
       <c r="F4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -904,8 +920,11 @@
       <c r="F5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -924,8 +943,11 @@
       <c r="F6" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -944,8 +966,11 @@
       <c r="F7" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -964,8 +989,11 @@
       <c r="F8" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -984,8 +1012,11 @@
       <c r="F9" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>50</v>
       </c>
@@ -1004,8 +1035,11 @@
       <c r="F10" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -1024,8 +1058,11 @@
       <c r="F11" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>58</v>
       </c>
@@ -1044,8 +1081,11 @@
       <c r="F12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>62</v>
       </c>
@@ -1063,6 +1103,9 @@
       </c>
       <c r="F13" t="s">
         <v>57</v>
+      </c>
+      <c r="G13">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor GUI validation and improve character loading
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -1177,17 +1177,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Сщщщщд</t>
+          <t>Cool</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Elf</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rogue</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1197,28 +1197,28 @@
         <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G2" t="n">
         <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I2" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="J2" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K2" t="n">
         <v>12</v>
       </c>
       <c r="L2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="M2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>